<commit_message>
fixes and updated plots
</commit_message>
<xml_diff>
--- a/les_data/sf_case_log.xlsx
+++ b/les_data/sf_case_log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannahwilliams/GoogleDrive_Princeton/Research/projects_and_data/spectrum_farms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F45FC99C-AD42-CA4E-BB3D-65880F6D7145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7349FC1-B944-7048-A434-7B53297C4851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14520" yWindow="660" windowWidth="14700" windowHeight="17180" xr2:uid="{5690398C-59F1-6347-BCC4-BBF38ABBA979}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="463">
   <si>
     <t>Case number</t>
   </si>
@@ -1363,9 +1363,6 @@
   </si>
   <si>
     <t>kp16_js_match</t>
-  </si>
-  <si>
-    <t>running rmp</t>
   </si>
   <si>
     <t>U24_HS04_js</t>
@@ -2244,13 +2241,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2317,113 +2314,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="46">
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD8FFD8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFAC6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9AA8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7C9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD8FFD8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFAC6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF9AA8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7C9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="39">
     <dxf>
       <fill>
         <patternFill>
@@ -2661,6 +2552,54 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7C9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD8FFD8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFAC6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9AA8"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7C9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5203,12 +5142,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="L1" s="174" t="s">
+      <c r="L1" s="175" t="s">
         <v>366</v>
       </c>
-      <c r="M1" s="174"/>
-      <c r="N1" s="174"/>
-      <c r="O1" s="174"/>
+      <c r="M1" s="175"/>
+      <c r="N1" s="175"/>
+      <c r="O1" s="175"/>
       <c r="P1" s="170"/>
       <c r="Q1" s="170"/>
       <c r="S1" s="135" t="s">
@@ -5219,12 +5158,12 @@
       <c r="V1" s="135"/>
       <c r="W1" s="135"/>
       <c r="X1" s="135"/>
-      <c r="AB1" s="175" t="s">
+      <c r="AB1" s="176" t="s">
         <v>367</v>
       </c>
-      <c r="AC1" s="175"/>
-      <c r="AD1" s="175"/>
-      <c r="AE1" s="175"/>
+      <c r="AC1" s="176"/>
+      <c r="AD1" s="176"/>
+      <c r="AE1" s="176"/>
     </row>
     <row r="2" spans="1:34" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="120" t="s">
@@ -7276,7 +7215,7 @@
     </row>
     <row r="24" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="121" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B24" s="116">
         <v>1.0369999999999999</v>
@@ -7377,7 +7316,7 @@
     </row>
     <row r="25" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="121" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B25" s="116">
         <v>0.65900000000000003</v>
@@ -7478,7 +7417,7 @@
     </row>
     <row r="26" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="121" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B26" s="116">
         <v>0.79900000000000004</v>
@@ -7579,7 +7518,7 @@
     </row>
     <row r="27" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="121" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B27" s="116">
         <v>1.0189999999999999</v>
@@ -7680,7 +7619,7 @@
     </row>
     <row r="28" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="121" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B28" s="116">
         <v>0.53</v>
@@ -7781,7 +7720,7 @@
     </row>
     <row r="29" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="121" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="B29" s="116">
         <v>0.32100000000000001</v>
@@ -7882,7 +7821,7 @@
     </row>
     <row r="30" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="121" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B30" s="116">
         <v>0.39500000000000002</v>
@@ -7983,7 +7922,7 @@
     </row>
     <row r="31" spans="1:34" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="121" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B31" s="116">
         <v>0.54400000000000004</v>
@@ -9046,7 +8985,7 @@
     </row>
     <row r="43" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="121" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B43">
         <v>0.72499999999999998</v>
@@ -9140,7 +9079,7 @@
     </row>
     <row r="44" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="121" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B44">
         <v>0.61899999999999999</v>
@@ -9234,7 +9173,7 @@
     </row>
     <row r="45" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="121" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B45">
         <v>0.82</v>
@@ -9328,7 +9267,7 @@
     </row>
     <row r="46" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="121" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B46">
         <v>0.65</v>
@@ -9422,7 +9361,7 @@
     </row>
     <row r="47" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="121" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B47">
         <v>0.91700000000000004</v>
@@ -9516,7 +9455,7 @@
     </row>
     <row r="48" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="121" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="B48">
         <v>0.92700000000000005</v>
@@ -9610,10 +9549,10 @@
     </row>
     <row r="49" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="121" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B49">
-        <v>0.96099999999999997</v>
+        <v>0.97099999999999997</v>
       </c>
       <c r="F49">
         <v>24</v>
@@ -9651,7 +9590,7 @@
         <v>10.292999999999999</v>
       </c>
       <c r="R49" s="116" t="s">
-        <v>439</v>
+        <v>31</v>
       </c>
       <c r="S49" s="116">
         <v>0.5</v>
@@ -9683,7 +9622,7 @@
       </c>
       <c r="AB49" s="123">
         <f t="shared" si="81"/>
-        <v>8.2254807403437873</v>
+        <v>8.1407693012053333</v>
       </c>
       <c r="AC49" s="123" t="e">
         <f t="shared" si="82"/>
@@ -9706,7 +9645,7 @@
     </row>
     <row r="50" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="121" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="B50">
         <v>0.96099999999999997</v>
@@ -9802,7 +9741,7 @@
     </row>
     <row r="51" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="121" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B51">
         <v>0.34</v>
@@ -9896,7 +9835,7 @@
     </row>
     <row r="52" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="121" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B52">
         <v>0.309</v>
@@ -9990,7 +9929,7 @@
     </row>
     <row r="53" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="121" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B53">
         <v>0.375</v>
@@ -10084,7 +10023,7 @@
     </row>
     <row r="54" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="121" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B54">
         <v>0.30299999999999999</v>
@@ -10178,7 +10117,7 @@
     </row>
     <row r="55" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="121" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B55">
         <v>0.497</v>
@@ -10272,7 +10211,7 @@
     </row>
     <row r="56" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="121" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B56">
         <v>0.45400000000000001</v>
@@ -10366,7 +10305,7 @@
     </row>
     <row r="57" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="121" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B57">
         <v>0.50600000000000001</v>
@@ -10462,7 +10401,7 @@
     </row>
     <row r="58" spans="1:33" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="121" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B58">
         <v>0.45700000000000002</v>
@@ -10564,26 +10503,26 @@
     <mergeCell ref="L1:O1"/>
     <mergeCell ref="AB1:AE1"/>
   </mergeCells>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="expression" dxfId="38" priority="1" stopIfTrue="1">
+      <formula>$R1="running rmp"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="37" priority="2">
+      <formula>$R1="running st"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="R3:R58">
-    <cfRule type="containsText" dxfId="11" priority="3" stopIfTrue="1" operator="containsText" text="bad">
+    <cfRule type="containsText" dxfId="36" priority="3" stopIfTrue="1" operator="containsText" text="bad">
       <formula>NOT(ISERROR(SEARCH("bad",R3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="4" stopIfTrue="1" operator="containsText" text="error">
+    <cfRule type="containsText" dxfId="35" priority="4" stopIfTrue="1" operator="containsText" text="error">
       <formula>NOT(ISERROR(SEARCH("error",R3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="5" stopIfTrue="1" operator="containsText" text="running">
+    <cfRule type="containsText" dxfId="34" priority="5" stopIfTrue="1" operator="containsText" text="running">
       <formula>NOT(ISERROR(SEARCH("running",R3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="done">
+    <cfRule type="containsText" dxfId="33" priority="6" operator="containsText" text="done">
       <formula>NOT(ISERROR(SEARCH("done",R3)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="expression" dxfId="6" priority="2">
-      <formula>$R1="running st"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="1" stopIfTrue="1">
-      <formula>$R1="running rmp"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12722,15 +12661,15 @@
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="Y1:Y1048576">
-    <cfRule type="containsText" dxfId="15" priority="1" operator="containsText" text=".">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text=".">
       <formula>NOT(ISERROR(SEARCH(".",Y1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y5:Y99">
-    <cfRule type="containsBlanks" dxfId="14" priority="2">
+    <cfRule type="containsBlanks" dxfId="1" priority="2">
       <formula>LEN(TRIM(Y5))=0</formula>
     </cfRule>
-    <cfRule type="notContainsText" dxfId="13" priority="3" operator="notContains" text="done">
+    <cfRule type="notContainsText" dxfId="0" priority="3" operator="notContains" text="done">
       <formula>ISERROR(SEARCH("done",Y5))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13478,19 +13417,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="K1" s="174" t="s">
+      <c r="K1" s="175" t="s">
         <v>366</v>
       </c>
-      <c r="L1" s="174"/>
-      <c r="M1" s="174"/>
-      <c r="N1" s="174"/>
-      <c r="P1" s="176" t="s">
+      <c r="L1" s="175"/>
+      <c r="M1" s="175"/>
+      <c r="N1" s="175"/>
+      <c r="P1" s="174" t="s">
         <v>366</v>
       </c>
-      <c r="Q1" s="176"/>
-      <c r="R1" s="176"/>
-      <c r="S1" s="176"/>
-      <c r="T1" s="176"/>
+      <c r="Q1" s="174"/>
+      <c r="R1" s="174"/>
+      <c r="S1" s="174"/>
+      <c r="T1" s="174"/>
     </row>
     <row r="2" spans="1:29" s="118" customFormat="1" ht="26" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="120" t="s">
@@ -14450,16 +14389,16 @@
     <mergeCell ref="P1:T1"/>
   </mergeCells>
   <conditionalFormatting sqref="O3:O11">
-    <cfRule type="containsText" dxfId="45" priority="1" stopIfTrue="1" operator="containsText" text="bad">
+    <cfRule type="containsText" dxfId="32" priority="1" stopIfTrue="1" operator="containsText" text="bad">
       <formula>NOT(ISERROR(SEARCH("bad",O3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="2" stopIfTrue="1" operator="containsText" text="error">
+    <cfRule type="containsText" dxfId="31" priority="2" stopIfTrue="1" operator="containsText" text="error">
       <formula>NOT(ISERROR(SEARCH("error",O3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="43" priority="3" stopIfTrue="1" operator="containsText" text="running">
+    <cfRule type="containsText" dxfId="30" priority="3" stopIfTrue="1" operator="containsText" text="running">
       <formula>NOT(ISERROR(SEARCH("running",O3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="42" priority="4" operator="containsText" text="done">
+    <cfRule type="containsText" dxfId="29" priority="4" operator="containsText" text="done">
       <formula>NOT(ISERROR(SEARCH("done",O3)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14481,20 +14420,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.2">
-      <c r="K1" s="174" t="s">
+      <c r="K1" s="175" t="s">
         <v>366</v>
       </c>
-      <c r="L1" s="174"/>
-      <c r="M1" s="174"/>
-      <c r="N1" s="174"/>
-      <c r="P1" s="176" t="s">
+      <c r="L1" s="175"/>
+      <c r="M1" s="175"/>
+      <c r="N1" s="175"/>
+      <c r="P1" s="174" t="s">
         <v>366</v>
       </c>
-      <c r="Q1" s="176"/>
-      <c r="R1" s="176"/>
-      <c r="S1" s="176"/>
-      <c r="T1" s="176"/>
-      <c r="U1" s="176"/>
+      <c r="Q1" s="174"/>
+      <c r="R1" s="174"/>
+      <c r="S1" s="174"/>
+      <c r="T1" s="174"/>
+      <c r="U1" s="174"/>
     </row>
     <row r="2" spans="1:30" s="118" customFormat="1" ht="26" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="120" t="s">
@@ -16293,16 +16232,16 @@
     <mergeCell ref="K1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="O3:O7 O12:O22">
-    <cfRule type="containsText" dxfId="41" priority="1" stopIfTrue="1" operator="containsText" text="bad">
+    <cfRule type="containsText" dxfId="28" priority="1" stopIfTrue="1" operator="containsText" text="bad">
       <formula>NOT(ISERROR(SEARCH("bad",O3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="40" priority="2" stopIfTrue="1" operator="containsText" text="error">
+    <cfRule type="containsText" dxfId="27" priority="2" stopIfTrue="1" operator="containsText" text="error">
       <formula>NOT(ISERROR(SEARCH("error",O3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="39" priority="3" stopIfTrue="1" operator="containsText" text="running">
+    <cfRule type="containsText" dxfId="26" priority="3" stopIfTrue="1" operator="containsText" text="running">
       <formula>NOT(ISERROR(SEARCH("running",O3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="38" priority="4" operator="containsText" text="done">
+    <cfRule type="containsText" dxfId="25" priority="4" operator="containsText" text="done">
       <formula>NOT(ISERROR(SEARCH("done",O3)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17883,15 +17822,15 @@
     <mergeCell ref="E3:G3"/>
   </mergeCells>
   <conditionalFormatting sqref="AA1:AA4 AA6:AA1048576">
-    <cfRule type="containsText" dxfId="37" priority="1" operator="containsText" text=".">
+    <cfRule type="containsText" dxfId="24" priority="1" operator="containsText" text=".">
       <formula>NOT(ISERROR(SEARCH(".",AA1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA7:AA49">
-    <cfRule type="containsBlanks" dxfId="36" priority="2">
+    <cfRule type="containsBlanks" dxfId="23" priority="2">
       <formula>LEN(TRIM(AA7))=0</formula>
     </cfRule>
-    <cfRule type="notContainsText" dxfId="35" priority="3" operator="notContains" text="done">
+    <cfRule type="notContainsText" dxfId="22" priority="3" operator="notContains" text="done">
       <formula>ISERROR(SEARCH("done",AA7))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19733,16 +19672,16 @@
     <sortCondition descending="1" ref="P2:P20"/>
   </sortState>
   <conditionalFormatting sqref="P2:P20">
-    <cfRule type="containsText" dxfId="34" priority="1" stopIfTrue="1" operator="containsText" text="bad">
+    <cfRule type="containsText" dxfId="21" priority="1" stopIfTrue="1" operator="containsText" text="bad">
       <formula>NOT(ISERROR(SEARCH("bad",P2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="33" priority="20" stopIfTrue="1" operator="containsText" text="error">
+    <cfRule type="containsText" dxfId="20" priority="20" stopIfTrue="1" operator="containsText" text="error">
       <formula>NOT(ISERROR(SEARCH("error",P2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="32" priority="21" stopIfTrue="1" operator="containsText" text="running">
+    <cfRule type="containsText" dxfId="19" priority="21" stopIfTrue="1" operator="containsText" text="running">
       <formula>NOT(ISERROR(SEARCH("running",P2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="22" operator="containsText" text="done">
+    <cfRule type="containsText" dxfId="18" priority="22" operator="containsText" text="done">
       <formula>NOT(ISERROR(SEARCH("done",P2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -22642,16 +22581,16 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="P2:P29">
-    <cfRule type="containsText" dxfId="30" priority="1" stopIfTrue="1" operator="containsText" text="bad">
+    <cfRule type="containsText" dxfId="17" priority="1" stopIfTrue="1" operator="containsText" text="bad">
       <formula>NOT(ISERROR(SEARCH("bad",P2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="29" priority="2" stopIfTrue="1" operator="containsText" text="error">
+    <cfRule type="containsText" dxfId="16" priority="2" stopIfTrue="1" operator="containsText" text="error">
       <formula>NOT(ISERROR(SEARCH("error",P2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="3" stopIfTrue="1" operator="containsText" text="running">
+    <cfRule type="containsText" dxfId="15" priority="3" stopIfTrue="1" operator="containsText" text="running">
       <formula>NOT(ISERROR(SEARCH("running",P2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="27" priority="4" operator="containsText" text="done">
+    <cfRule type="containsText" dxfId="14" priority="4" operator="containsText" text="done">
       <formula>NOT(ISERROR(SEARCH("done",P2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -24016,16 +23955,16 @@
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="L2:L22">
-    <cfRule type="containsText" dxfId="26" priority="1" stopIfTrue="1" operator="containsText" text="bad">
+    <cfRule type="containsText" dxfId="13" priority="1" stopIfTrue="1" operator="containsText" text="bad">
       <formula>NOT(ISERROR(SEARCH("bad",L2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="25" priority="2" stopIfTrue="1" operator="containsText" text="error">
+    <cfRule type="containsText" dxfId="12" priority="2" stopIfTrue="1" operator="containsText" text="error">
       <formula>NOT(ISERROR(SEARCH("error",L2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="3" stopIfTrue="1" operator="containsText" text="running">
+    <cfRule type="containsText" dxfId="11" priority="3" stopIfTrue="1" operator="containsText" text="running">
       <formula>NOT(ISERROR(SEARCH("running",L2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="4" operator="containsText" text="done">
+    <cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="done">
       <formula>NOT(ISERROR(SEARCH("done",L2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -26639,16 +26578,16 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="N2:N29">
-    <cfRule type="containsText" dxfId="22" priority="1" stopIfTrue="1" operator="containsText" text="bad">
+    <cfRule type="containsText" dxfId="9" priority="1" stopIfTrue="1" operator="containsText" text="bad">
       <formula>NOT(ISERROR(SEARCH("bad",N2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="2" stopIfTrue="1" operator="containsText" text="error">
+    <cfRule type="containsText" dxfId="8" priority="2" stopIfTrue="1" operator="containsText" text="error">
       <formula>NOT(ISERROR(SEARCH("error",N2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="3" stopIfTrue="1" operator="containsText" text="running">
+    <cfRule type="containsText" dxfId="7" priority="3" stopIfTrue="1" operator="containsText" text="running">
       <formula>NOT(ISERROR(SEARCH("running",N2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="4" operator="containsText" text="done">
+    <cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="done">
       <formula>NOT(ISERROR(SEARCH("done",N2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -30347,15 +30286,15 @@
     <mergeCell ref="AA4:AF4"/>
   </mergeCells>
   <conditionalFormatting sqref="AJ1:AJ3 AJ5:AJ1048576">
-    <cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text=".">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text=".">
       <formula>NOT(ISERROR(SEARCH(".",AJ1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ6:AJ70">
-    <cfRule type="containsBlanks" dxfId="17" priority="2">
+    <cfRule type="containsBlanks" dxfId="4" priority="2">
       <formula>LEN(TRIM(AJ6))=0</formula>
     </cfRule>
-    <cfRule type="notContainsText" dxfId="16" priority="3" operator="notContains" text="done">
+    <cfRule type="notContainsText" dxfId="3" priority="3" operator="notContains" text="done">
       <formula>ISERROR(SEARCH("done",AJ6))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>